<commit_message>
Add Category entity, config, seeder, and mapping
Introduced Category entity with EF Core configuration and AutoMapper mapping. Registered Categories DbSet in AgricultureDbContext. Implemented CategorySeeder to import data from AgricultureData.xlsx and updated DataSeeder to include it. Updated Excel seed data file.
</commit_message>
<xml_diff>
--- a/src/External/Agriculture.Persistence/Data/AgricultureData.xlsx
+++ b/src/External/Agriculture.Persistence/Data/AgricultureData.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30306"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="67" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{669C12EE-2E2F-40A2-A120-5A864F7F587F}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1592BAA-1886-45EC-8BFD-17DC4705704F}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PlantSpecices" sheetId="1" r:id="rId1"/>
+    <sheet name="Categories" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="60">
   <si>
     <t>Id</t>
   </si>
@@ -154,6 +155,66 @@
   </si>
   <si>
     <t>Perennial fruit plant producing sweet berries.</t>
+  </si>
+  <si>
+    <t>Vegetable</t>
+  </si>
+  <si>
+    <t>Rau</t>
+  </si>
+  <si>
+    <t>Fruit</t>
+  </si>
+  <si>
+    <t>Cây ăn quả</t>
+  </si>
+  <si>
+    <t>Flower</t>
+  </si>
+  <si>
+    <t>Hoa</t>
+  </si>
+  <si>
+    <t>Herb</t>
+  </si>
+  <si>
+    <t>Rau thơm</t>
+  </si>
+  <si>
+    <t>Grain</t>
+  </si>
+  <si>
+    <t>Ngũ cốc</t>
+  </si>
+  <si>
+    <t>Legume</t>
+  </si>
+  <si>
+    <t>Cây họ đậu</t>
+  </si>
+  <si>
+    <t>Spice</t>
+  </si>
+  <si>
+    <t>Gia vị</t>
+  </si>
+  <si>
+    <t>Medicinal</t>
+  </si>
+  <si>
+    <t>Cây dược liệu</t>
+  </si>
+  <si>
+    <t>Ornamental</t>
+  </si>
+  <si>
+    <t>Cây cảnh</t>
+  </si>
+  <si>
+    <t>Mushroom</t>
+  </si>
+  <si>
+    <t>Nấm</t>
   </si>
 </sst>
 </file>
@@ -881,4 +942,138 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4F0ABE6-3D17-4276-AE94-5346E81A68FE}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add garden and plot seeding with unique plot index
- Added GardenSeeder and GardenPlotSeeder to seed data from AgricultureData.xlsx using MiniExcel.
- Enforced unique (GardenId, Row, Column) index in GardenPlotConfiguration.
- Renamed GardentPlotResponse to GardenPlotResponse and updated mappings.
- Registered new seeders in DataSeeder.
- Updated GardenResponse and mapping profiles accordingly.
- Updated AgricultureData.xlsx with seed data.
</commit_message>
<xml_diff>
--- a/src/External/Agriculture.Persistence/Data/AgricultureData.xlsx
+++ b/src/External/Agriculture.Persistence/Data/AgricultureData.xlsx
@@ -1,15 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30306"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30309"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="80" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1592BAA-1886-45EC-8BFD-17DC4705704F}"/>
+  <xr:revisionPtr revIDLastSave="104" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C7B6F2A-5D12-49D0-842F-9B298ACEB1DE}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PlantSpecices" sheetId="1" r:id="rId1"/>
     <sheet name="Categories" sheetId="2" r:id="rId2"/>
+    <sheet name="Gardens" sheetId="3" r:id="rId3"/>
+    <sheet name="GardenPlots" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="80">
   <si>
     <t>Id</t>
   </si>
@@ -215,6 +217,66 @@
   </si>
   <si>
     <t>Nấm</t>
+  </si>
+  <si>
+    <t>Home Garden</t>
+  </si>
+  <si>
+    <t>Small backyard garden for vegetables and herbs.</t>
+  </si>
+  <si>
+    <t>Green Valley Farm</t>
+  </si>
+  <si>
+    <t>Large outdoor farming area for seasonal crops.</t>
+  </si>
+  <si>
+    <t>Sunny Orchard</t>
+  </si>
+  <si>
+    <t>Garden specializing in fruit trees.</t>
+  </si>
+  <si>
+    <t>Urban Rooftop</t>
+  </si>
+  <si>
+    <t>Rooftop garden with raised planting beds.</t>
+  </si>
+  <si>
+    <t>Tropical Paradise</t>
+  </si>
+  <si>
+    <t>Garden for tropical fruits and flowers.</t>
+  </si>
+  <si>
+    <t>GardenId</t>
+  </si>
+  <si>
+    <t>Row</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>SoilType</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Loam</t>
+  </si>
+  <si>
+    <t>Empty</t>
+  </si>
+  <si>
+    <t>Sandy</t>
+  </si>
+  <si>
+    <t>Clay</t>
+  </si>
+  <si>
+    <t>Silt</t>
   </si>
 </sst>
 </file>
@@ -1076,4 +1138,594 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A11C1940-CD17-44E2-959E-2D499BAD76F5}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1A2F1B1-7FBC-4294-99D0-449C26FC6460}">
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>79</v>
+      </c>
+      <c r="F9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" t="s">
+        <v>77</v>
+      </c>
+      <c r="F12" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>2</v>
+      </c>
+      <c r="E13" t="s">
+        <v>75</v>
+      </c>
+      <c r="F13" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>2</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
+        <v>78</v>
+      </c>
+      <c r="F14" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="E15" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>4</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>4</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>2</v>
+      </c>
+      <c r="E17" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>4</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>4</v>
+      </c>
+      <c r="C19">
+        <v>2</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>5</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20" t="s">
+        <v>79</v>
+      </c>
+      <c r="F20" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>5</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>2</v>
+      </c>
+      <c r="E21" t="s">
+        <v>75</v>
+      </c>
+      <c r="F21" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>5</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
+        <v>3</v>
+      </c>
+      <c r="E22" t="s">
+        <v>77</v>
+      </c>
+      <c r="F22" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>5</v>
+      </c>
+      <c r="C23">
+        <v>2</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23" t="s">
+        <v>78</v>
+      </c>
+      <c r="F23" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>5</v>
+      </c>
+      <c r="C24">
+        <v>2</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="E24" t="s">
+        <v>75</v>
+      </c>
+      <c r="F24" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>5</v>
+      </c>
+      <c r="C25">
+        <v>2</v>
+      </c>
+      <c r="D25">
+        <v>3</v>
+      </c>
+      <c r="E25" t="s">
+        <v>79</v>
+      </c>
+      <c r="F25" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Garden Template feature with API and data refactor
Introduces GardenTemplate and GardenPlotTemplate entities, DTOs, repository, service, and API endpoints for managing reusable garden layouts. Replaces static garden/plot seeders with template-based seeders, updates dependency injection and DbContext, and adds MediatR queries/handlers. Existing DTOs updated with PublicId fields. Excel seed data updated for templates. Removes legacy garden/plot seeders and mappings.
</commit_message>
<xml_diff>
--- a/src/External/Agriculture.Persistence/Data/AgricultureData.xlsx
+++ b/src/External/Agriculture.Persistence/Data/AgricultureData.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30305"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="104" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C7B6F2A-5D12-49D0-842F-9B298ACEB1DE}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{042BFCA7-03C4-49C6-B1F3-8115BCD24260}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PlantSpecices" sheetId="1" r:id="rId1"/>
     <sheet name="Categories" sheetId="2" r:id="rId2"/>
-    <sheet name="Gardens" sheetId="3" r:id="rId3"/>
-    <sheet name="GardenPlots" sheetId="4" r:id="rId4"/>
+    <sheet name="GardenTemplates" sheetId="3" r:id="rId3"/>
+    <sheet name="GardenPlotTemplates" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="85">
   <si>
     <t>Id</t>
   </si>
@@ -219,18 +219,36 @@
     <t>Nấm</t>
   </si>
   <si>
+    <t>UnlockType</t>
+  </si>
+  <si>
+    <t>UnlockValue</t>
+  </si>
+  <si>
+    <t>UnlockPrice</t>
+  </si>
+  <si>
+    <t>ReferenceId</t>
+  </si>
+  <si>
     <t>Home Garden</t>
   </si>
   <si>
     <t>Small backyard garden for vegetables and herbs.</t>
   </si>
   <si>
+    <t>None</t>
+  </si>
+  <si>
     <t>Green Valley Farm</t>
   </si>
   <si>
     <t>Large outdoor farming area for seasonal crops.</t>
   </si>
   <si>
+    <t>Level</t>
+  </si>
+  <si>
     <t>Sunny Orchard</t>
   </si>
   <si>
@@ -243,13 +261,16 @@
     <t>Rooftop garden with raised planting beds.</t>
   </si>
   <si>
+    <t>Purchase</t>
+  </si>
+  <si>
     <t>Tropical Paradise</t>
   </si>
   <si>
     <t>Garden for tropical fruits and flowers.</t>
   </si>
   <si>
-    <t>GardenId</t>
+    <t>GardenTemplateId</t>
   </si>
   <si>
     <t>Row</t>
@@ -261,13 +282,7 @@
     <t>SoilType</t>
   </si>
   <si>
-    <t>Status</t>
-  </si>
-  <si>
     <t>Loam</t>
-  </si>
-  <si>
-    <t>Empty</t>
   </si>
   <si>
     <t>Sandy</t>
@@ -1141,15 +1156,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A11C1940-CD17-44E2-959E-2D499BAD76F5}">
-  <dimension ref="A1:C6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BD73BF2-BA09-498D-A62C-AFD6E043259B}">
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="44.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1159,60 +1176,117 @@
       <c r="C1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>65</v>
+      </c>
+      <c r="D2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+        <v>68</v>
+      </c>
+      <c r="D3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="F3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+        <v>71</v>
+      </c>
+      <c r="D4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4">
+        <v>10</v>
+      </c>
+      <c r="F4">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <v>73</v>
+      </c>
+      <c r="D5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
+        <v>76</v>
+      </c>
+      <c r="D6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>12000</v>
       </c>
     </row>
   </sheetData>
@@ -1221,31 +1295,28 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1A2F1B1-7FBC-4294-99D0-449C26FC6460}">
-  <dimension ref="A1:F25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78E00C35-E09E-4E6F-B62E-E7FD80572362}">
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="E1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1259,13 +1330,10 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>75</v>
-      </c>
-      <c r="F2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1279,13 +1347,10 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1299,13 +1364,10 @@
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>77</v>
-      </c>
-      <c r="F4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1319,13 +1381,10 @@
         <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F5" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1339,13 +1398,10 @@
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>75</v>
-      </c>
-      <c r="F6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1359,13 +1415,10 @@
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F7" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1379,13 +1432,10 @@
         <v>3</v>
       </c>
       <c r="E8" t="s">
-        <v>77</v>
-      </c>
-      <c r="F8" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1399,13 +1449,10 @@
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>79</v>
-      </c>
-      <c r="F9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1419,13 +1466,10 @@
         <v>2</v>
       </c>
       <c r="E10" t="s">
-        <v>78</v>
-      </c>
-      <c r="F10" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1439,13 +1483,10 @@
         <v>3</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
-      </c>
-      <c r="F11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1459,13 +1500,10 @@
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>77</v>
-      </c>
-      <c r="F12" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1479,13 +1517,10 @@
         <v>2</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
-      </c>
-      <c r="F13" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1499,13 +1534,10 @@
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>78</v>
-      </c>
-      <c r="F14" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1519,13 +1551,10 @@
         <v>2</v>
       </c>
       <c r="E15" t="s">
-        <v>79</v>
-      </c>
-      <c r="F15" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1539,13 +1568,10 @@
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>75</v>
-      </c>
-      <c r="F16" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1559,13 +1585,10 @@
         <v>2</v>
       </c>
       <c r="E17" t="s">
-        <v>77</v>
-      </c>
-      <c r="F17" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1579,13 +1602,10 @@
         <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>78</v>
-      </c>
-      <c r="F18" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1599,13 +1619,10 @@
         <v>2</v>
       </c>
       <c r="E19" t="s">
-        <v>75</v>
-      </c>
-      <c r="F19" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1619,13 +1636,10 @@
         <v>1</v>
       </c>
       <c r="E20" t="s">
-        <v>79</v>
-      </c>
-      <c r="F20" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1639,13 +1653,10 @@
         <v>2</v>
       </c>
       <c r="E21" t="s">
-        <v>75</v>
-      </c>
-      <c r="F21" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1659,13 +1670,10 @@
         <v>3</v>
       </c>
       <c r="E22" t="s">
-        <v>77</v>
-      </c>
-      <c r="F22" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1679,13 +1687,10 @@
         <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>78</v>
-      </c>
-      <c r="F23" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1699,13 +1704,10 @@
         <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>75</v>
-      </c>
-      <c r="F24" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1719,10 +1721,7 @@
         <v>3</v>
       </c>
       <c r="E25" t="s">
-        <v>79</v>
-      </c>
-      <c r="F25" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor Category/Plant relationships and update configs
- Category now relates to PlantSpecices, not Plants; PlantSpecices references Category.
- Removed Category reference from Plant; Plant now references PlantSpecices.
- Added Plant navigation to GardenPlot.
- Updated EF Core configurations for new relationships and constraints.
- Added PlantConfiguration for Plant entity mapping.
- Updated seeders and AgricultureData.xlsx for new structure.
- Adjusted DbSet properties and constructors as needed.
</commit_message>
<xml_diff>
--- a/src/External/Agriculture.Persistence/Data/AgricultureData.xlsx
+++ b/src/External/Agriculture.Persistence/Data/AgricultureData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30305"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="164" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{042BFCA7-03C4-49C6-B1F3-8115BCD24260}"/>
+  <xr:revisionPtr revIDLastSave="200" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C46355B-F871-4A21-9927-0887643FF5C6}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PlantSpecices" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="86">
   <si>
     <t>Id</t>
   </si>
@@ -67,6 +67,9 @@
   </si>
   <si>
     <t>TemperatureMax</t>
+  </si>
+  <si>
+    <t>CategoryId</t>
   </si>
   <si>
     <t>Tomato</t>
@@ -650,7 +653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
@@ -664,7 +667,7 @@
     <col min="10" max="10" width="16.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -695,19 +698,22 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" s="1">
         <v>30</v>
@@ -727,19 +733,22 @@
       <c r="J2" s="1">
         <v>30</v>
       </c>
-    </row>
-    <row r="3" spans="1:10">
+      <c r="K2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E3" s="1">
         <v>20</v>
@@ -759,19 +768,22 @@
       <c r="J3" s="1">
         <v>24</v>
       </c>
-    </row>
-    <row r="4" spans="1:10">
+      <c r="K3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" s="1">
         <v>35</v>
@@ -791,19 +803,22 @@
       <c r="J4" s="1">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:10">
+      <c r="K4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E5" s="1">
         <v>25</v>
@@ -823,19 +838,22 @@
       <c r="J5" s="1">
         <v>30</v>
       </c>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" s="1">
         <v>35</v>
@@ -855,19 +873,22 @@
       <c r="J6" s="1">
         <v>32</v>
       </c>
-    </row>
-    <row r="7" spans="1:10">
+      <c r="K6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E7" s="1">
         <v>18</v>
@@ -887,19 +908,22 @@
       <c r="J7" s="1">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:10">
+      <c r="K7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E8" s="1">
         <v>30</v>
@@ -919,19 +943,22 @@
       <c r="J8" s="1">
         <v>24</v>
       </c>
-    </row>
-    <row r="9" spans="1:10">
+      <c r="K8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E9" s="1">
         <v>45</v>
@@ -951,19 +978,22 @@
       <c r="J9" s="1">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:10">
+      <c r="K9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E10" s="1">
         <v>20</v>
@@ -983,19 +1013,22 @@
       <c r="J10" s="1">
         <v>32</v>
       </c>
-    </row>
-    <row r="11" spans="1:10">
+      <c r="K10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E11" s="1">
         <v>35</v>
@@ -1014,6 +1047,9 @@
       </c>
       <c r="J11" s="1">
         <v>28</v>
+      </c>
+      <c r="K11">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1045,10 +1081,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1056,10 +1092,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1067,10 +1103,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1078,10 +1114,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1089,10 +1125,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1100,10 +1136,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1111,10 +1147,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1122,10 +1158,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1133,10 +1169,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1144,10 +1180,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1177,16 +1213,16 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -1194,13 +1230,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1214,13 +1250,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E3">
         <v>5</v>
@@ -1234,13 +1270,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" t="s">
         <v>70</v>
-      </c>
-      <c r="C4" t="s">
-        <v>71</v>
-      </c>
-      <c r="D4" t="s">
-        <v>69</v>
       </c>
       <c r="E4">
         <v>10</v>
@@ -1254,13 +1290,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1274,13 +1310,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" t="s">
         <v>75</v>
-      </c>
-      <c r="C6" t="s">
-        <v>76</v>
-      </c>
-      <c r="D6" t="s">
-        <v>74</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1304,16 +1340,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1330,7 +1366,7 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1347,7 +1383,7 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1364,7 +1400,7 @@
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1381,7 +1417,7 @@
         <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1398,7 +1434,7 @@
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1415,7 +1451,7 @@
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1432,7 +1468,7 @@
         <v>3</v>
       </c>
       <c r="E8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1449,7 +1485,7 @@
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1466,7 +1502,7 @@
         <v>2</v>
       </c>
       <c r="E10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1483,7 +1519,7 @@
         <v>3</v>
       </c>
       <c r="E11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1500,7 +1536,7 @@
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1517,7 +1553,7 @@
         <v>2</v>
       </c>
       <c r="E13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1534,7 +1570,7 @@
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1551,7 +1587,7 @@
         <v>2</v>
       </c>
       <c r="E15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1568,7 +1604,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1585,7 +1621,7 @@
         <v>2</v>
       </c>
       <c r="E17" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1602,7 +1638,7 @@
         <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1619,7 +1655,7 @@
         <v>2</v>
       </c>
       <c r="E19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1636,7 +1672,7 @@
         <v>1</v>
       </c>
       <c r="E20" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1653,7 +1689,7 @@
         <v>2</v>
       </c>
       <c r="E21" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1670,7 +1706,7 @@
         <v>3</v>
       </c>
       <c r="E22" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1687,7 +1723,7 @@
         <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1704,7 +1740,7 @@
         <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1721,7 +1757,7 @@
         <v>3</v>
       </c>
       <c r="E25" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add planting feature and role seeder to API
Introduce POST /api/plants/planting endpoint with PlantRequest DTO and MediatR command/handler for planting logic. Update Plant entity (nullable HarvestAt, constructors, expected harvest logic). Enhance specifications for eager loading. Add PlantAsync to IPlantService and implementation. Extend repositories with FindAsync methods. Update AutoMapper profiles. Add RoleSeeder for Excel-based role seeding and integrate into main seeder. Include minor fixes and mapping corrections.
</commit_message>
<xml_diff>
--- a/src/External/Agriculture.Persistence/Data/AgricultureData.xlsx
+++ b/src/External/Agriculture.Persistence/Data/AgricultureData.xlsx
@@ -3,15 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30305"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="200" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C46355B-F871-4A21-9927-0887643FF5C6}"/>
+  <xr:revisionPtr revIDLastSave="211" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDB84450-DACA-4C24-9358-BE568F20D238}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PlantSpecices" sheetId="1" r:id="rId1"/>
-    <sheet name="Categories" sheetId="2" r:id="rId2"/>
-    <sheet name="GardenTemplates" sheetId="3" r:id="rId3"/>
-    <sheet name="GardenPlotTemplates" sheetId="4" r:id="rId4"/>
+    <sheet name="Roles" sheetId="5" r:id="rId2"/>
+    <sheet name="Categories" sheetId="2" r:id="rId3"/>
+    <sheet name="GardenTemplates" sheetId="3" r:id="rId4"/>
+    <sheet name="GardenPlotTemplates" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="88">
   <si>
     <t>Id</t>
   </si>
@@ -160,6 +161,12 @@
   </si>
   <si>
     <t>Perennial fruit plant producing sweet berries.</t>
+  </si>
+  <si>
+    <t>Player</t>
+  </si>
+  <si>
+    <t>Admin</t>
   </si>
   <si>
     <t>Vegetable</t>
@@ -1058,6 +1065,43 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{510087A7-1D37-435C-AA06-D1E7424047C4}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4F0ABE6-3D17-4276-AE94-5346E81A68FE}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1081,10 +1125,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1092,10 +1136,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1103,10 +1147,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1114,10 +1158,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1125,10 +1169,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1136,10 +1180,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1147,10 +1191,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1158,10 +1202,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1169,10 +1213,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1180,10 +1224,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1191,7 +1235,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BD73BF2-BA09-498D-A62C-AFD6E043259B}">
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1213,16 +1257,16 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -1230,13 +1274,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1250,13 +1294,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E3">
         <v>5</v>
@@ -1270,13 +1314,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4" t="s">
         <v>72</v>
-      </c>
-      <c r="D4" t="s">
-        <v>70</v>
       </c>
       <c r="E4">
         <v>10</v>
@@ -1290,13 +1334,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1310,13 +1354,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" t="s">
         <v>77</v>
-      </c>
-      <c r="D6" t="s">
-        <v>75</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1330,7 +1374,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78E00C35-E09E-4E6F-B62E-E7FD80572362}">
   <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1340,16 +1384,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1366,7 +1410,7 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1383,7 +1427,7 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1400,7 +1444,7 @@
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1417,7 +1461,7 @@
         <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1434,7 +1478,7 @@
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1451,7 +1495,7 @@
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1468,7 +1512,7 @@
         <v>3</v>
       </c>
       <c r="E8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1485,7 +1529,7 @@
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1502,7 +1546,7 @@
         <v>2</v>
       </c>
       <c r="E10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1519,7 +1563,7 @@
         <v>3</v>
       </c>
       <c r="E11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1536,7 +1580,7 @@
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1553,7 +1597,7 @@
         <v>2</v>
       </c>
       <c r="E13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1570,7 +1614,7 @@
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1587,7 +1631,7 @@
         <v>2</v>
       </c>
       <c r="E15" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1604,7 +1648,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1621,7 +1665,7 @@
         <v>2</v>
       </c>
       <c r="E17" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1638,7 +1682,7 @@
         <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1655,7 +1699,7 @@
         <v>2</v>
       </c>
       <c r="E19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1672,7 +1716,7 @@
         <v>1</v>
       </c>
       <c r="E20" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1689,7 +1733,7 @@
         <v>2</v>
       </c>
       <c r="E21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1706,7 +1750,7 @@
         <v>3</v>
       </c>
       <c r="E22" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1723,7 +1767,7 @@
         <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1740,7 +1784,7 @@
         <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1757,7 +1801,7 @@
         <v>3</v>
       </c>
       <c r="E25" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>